<commit_message>
update on rules and csv
</commit_message>
<xml_diff>
--- a/surgical_staging/STAGED_CRS620MI_Suppliers.xlsx
+++ b/surgical_staging/STAGED_CRS620MI_Suppliers.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="122">
   <si>
     <t>IDCONO</t>
   </si>
@@ -130,6 +130,9 @@
     <t xml:space="preserve">500970    </t>
   </si>
   <si>
+    <t xml:space="preserve">501013    </t>
+  </si>
+  <si>
     <t xml:space="preserve">501023    </t>
   </si>
   <si>
@@ -151,6 +154,9 @@
     <t xml:space="preserve">Soarus, L.L.C.                      </t>
   </si>
   <si>
+    <t xml:space="preserve">Stonhard                            </t>
+  </si>
+  <si>
     <t xml:space="preserve">Sun Chemical Corp                   </t>
   </si>
   <si>
@@ -169,6 +175,9 @@
     <t xml:space="preserve">SOARUS    </t>
   </si>
   <si>
+    <t xml:space="preserve">STONHARD  </t>
+  </si>
+  <si>
     <t xml:space="preserve">SUN CHEM  </t>
   </si>
   <si>
@@ -184,6 +193,9 @@
     <t xml:space="preserve">           </t>
   </si>
   <si>
+    <t xml:space="preserve">560184790  </t>
+  </si>
+  <si>
     <t xml:space="preserve">222761297  </t>
   </si>
   <si>
@@ -208,6 +220,9 @@
     <t xml:space="preserve">(847) 255-1211  </t>
   </si>
   <si>
+    <t xml:space="preserve">(770) 425-9215  </t>
+  </si>
+  <si>
     <t xml:space="preserve">(404) 355-4131  </t>
   </si>
   <si>
@@ -226,6 +241,9 @@
     <t xml:space="preserve">(847) 255-4343  </t>
   </si>
   <si>
+    <t xml:space="preserve">(770) 425-6215  </t>
+  </si>
+  <si>
     <t xml:space="preserve">(404) 355-8741  </t>
   </si>
   <si>
@@ -298,6 +316,9 @@
     <t>141519.0</t>
   </si>
   <si>
+    <t>141523.0</t>
+  </si>
+  <si>
     <t>141524.0</t>
   </si>
   <si>
@@ -316,6 +337,9 @@
     <t>20230814.0</t>
   </si>
   <si>
+    <t>20050127.0</t>
+  </si>
+  <si>
     <t>20251204.0</t>
   </si>
   <si>
@@ -331,6 +355,9 @@
     <t>90.0</t>
   </si>
   <si>
+    <t>75.0</t>
+  </si>
+  <si>
     <t>83.0</t>
   </si>
   <si>
@@ -344,6 +371,9 @@
   </si>
   <si>
     <t xml:space="preserve">W20ACCAE  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">W20ACSNE  </t>
   </si>
   <si>
     <t xml:space="preserve">W70MEFOR  </t>
@@ -707,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AH8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:34">
@@ -822,100 +852,100 @@
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="O2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="P2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="Q2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="S2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="T2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="V2" t="s">
+        <v>89</v>
+      </c>
+      <c r="W2" t="s">
         <v>83</v>
       </c>
-      <c r="W2" t="s">
-        <v>77</v>
-      </c>
       <c r="X2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Y2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="Z2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="AA2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="AB2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="AC2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AD2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AE2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AF2" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="AG2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="AH2" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:34">
@@ -926,100 +956,100 @@
         <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="N3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="P3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="Q3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="S3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="T3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="V3" t="s">
+        <v>89</v>
+      </c>
+      <c r="W3" t="s">
         <v>83</v>
       </c>
-      <c r="W3" t="s">
-        <v>77</v>
-      </c>
       <c r="X3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Y3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="Z3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="AA3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="AB3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="AC3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AD3" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="AE3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="AF3" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="AG3" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="AH3" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:34">
@@ -1030,100 +1060,100 @@
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="K4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="N4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="O4" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="P4" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="Q4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R4" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="S4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="T4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W4" t="s">
+        <v>83</v>
+      </c>
+      <c r="X4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>85</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA4" t="s">
         <v>82</v>
       </c>
-      <c r="V4" t="s">
-        <v>83</v>
-      </c>
-      <c r="W4" t="s">
-        <v>77</v>
-      </c>
-      <c r="X4" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>76</v>
-      </c>
       <c r="AB4" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="AC4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AD4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AE4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="AF4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="AG4" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="AH4" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:34">
@@ -1134,100 +1164,100 @@
         <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="K5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="N5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="O5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="P5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="Q5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="S5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="T5" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U5" t="s">
+        <v>88</v>
+      </c>
+      <c r="V5" t="s">
+        <v>89</v>
+      </c>
+      <c r="W5" t="s">
+        <v>83</v>
+      </c>
+      <c r="X5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>85</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA5" t="s">
         <v>82</v>
       </c>
-      <c r="V5" t="s">
-        <v>83</v>
-      </c>
-      <c r="W5" t="s">
-        <v>77</v>
-      </c>
-      <c r="X5" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>76</v>
-      </c>
       <c r="AB5" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="AC5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AD5" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AE5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="AF5" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="AG5" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="AH5" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:34">
@@ -1238,100 +1268,100 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="K6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M6" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="N6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="O6" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="P6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="Q6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R6" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="S6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="T6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U6" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="V6" t="s">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="W6" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="X6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Y6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Z6" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="AA6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="AB6" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="AC6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AD6" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="AE6" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="AF6" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="AG6" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="AH6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:34">
@@ -1342,100 +1372,204 @@
         <v>40</v>
       </c>
       <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I7" t="s">
+        <v>64</v>
+      </c>
+      <c r="J7" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" t="s">
+        <v>71</v>
+      </c>
+      <c r="L7" t="s">
+        <v>71</v>
+      </c>
+      <c r="M7" t="s">
+        <v>71</v>
+      </c>
+      <c r="N7" t="s">
+        <v>79</v>
+      </c>
+      <c r="O7" t="s">
+        <v>80</v>
+      </c>
+      <c r="P7" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>71</v>
+      </c>
+      <c r="R7" t="s">
+        <v>83</v>
+      </c>
+      <c r="S7" t="s">
+        <v>85</v>
+      </c>
+      <c r="T7" t="s">
+        <v>86</v>
+      </c>
+      <c r="U7" t="s">
+        <v>87</v>
+      </c>
+      <c r="V7" t="s">
+        <v>42</v>
+      </c>
+      <c r="W7" t="s">
+        <v>83</v>
+      </c>
+      <c r="X7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>96</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>102</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>109</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" t="s">
-        <v>54</v>
-      </c>
-      <c r="G7" t="s">
-        <v>55</v>
-      </c>
-      <c r="H7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" t="s">
-        <v>59</v>
-      </c>
-      <c r="J7" t="s">
-        <v>66</v>
-      </c>
-      <c r="K7" t="s">
-        <v>66</v>
-      </c>
-      <c r="L7" t="s">
-        <v>66</v>
-      </c>
-      <c r="M7" t="s">
-        <v>66</v>
-      </c>
-      <c r="N7" t="s">
-        <v>71</v>
-      </c>
-      <c r="O7" t="s">
-        <v>74</v>
-      </c>
-      <c r="P7" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>66</v>
-      </c>
-      <c r="R7" t="s">
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" t="s">
+        <v>71</v>
+      </c>
+      <c r="K8" t="s">
+        <v>71</v>
+      </c>
+      <c r="L8" t="s">
+        <v>71</v>
+      </c>
+      <c r="M8" t="s">
+        <v>71</v>
+      </c>
+      <c r="N8" t="s">
         <v>77</v>
       </c>
-      <c r="S7" t="s">
-        <v>79</v>
-      </c>
-      <c r="T7" t="s">
+      <c r="O8" t="s">
         <v>80</v>
       </c>
-      <c r="U7" t="s">
-        <v>81</v>
-      </c>
-      <c r="V7" t="s">
-        <v>41</v>
-      </c>
-      <c r="W7" t="s">
-        <v>77</v>
-      </c>
-      <c r="X7" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>84</v>
-      </c>
-      <c r="Z7" t="s">
+      <c r="P8" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>71</v>
+      </c>
+      <c r="R8" t="s">
+        <v>83</v>
+      </c>
+      <c r="S8" t="s">
         <v>85</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="T8" t="s">
         <v>86</v>
       </c>
-      <c r="AB7" t="s">
+      <c r="U8" t="s">
         <v>87</v>
       </c>
-      <c r="AC7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AD7" t="s">
+      <c r="V8" t="s">
+        <v>42</v>
+      </c>
+      <c r="W8" t="s">
+        <v>83</v>
+      </c>
+      <c r="X8" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z8" t="s">
         <v>91</v>
       </c>
-      <c r="AE7" t="s">
-        <v>96</v>
-      </c>
-      <c r="AF7" t="s">
-        <v>91</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>106</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>111</v>
+      <c r="AA8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>97</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>97</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>